<commit_message>
correction of a typo
</commit_message>
<xml_diff>
--- a/earlyMBNMA-Forest_Plots/Time-course Adjusted Results at Week 24/Table_02_MG_ADL_score_change_from_baseline.xlsx
+++ b/earlyMBNMA-Forest_Plots/Time-course Adjusted Results at Week 24/Table_02_MG_ADL_score_change_from_baseline.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ebmhealth-my.sharepoint.com/personal/ananda_biswas_ebmhealth_in/Documents/Documents/R-Programs/earlyMBNMA-Forest_Plots/Time-course Adjusted Results at Week 24/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{BA390DF2-4AA3-453B-BE52-5A71AAC82B78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A612E31E-BD21-41DC-AA52-B21F86C85EFD}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="8_{BA390DF2-4AA3-453B-BE52-5A71AAC82B78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BCFE0E3F-5195-42FC-8760-901D3EC9C443}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3BB26D7E-CDC6-4541-AC86-3B29E419C628}"/>
   </bookViews>
@@ -634,10 +634,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1223,7 +1219,7 @@
         <v>-0.98</v>
       </c>
       <c r="C19" s="1">
-        <v>-2.91</v>
+        <v>-2.9</v>
       </c>
       <c r="D19" s="1">
         <v>1.01</v>

</xml_diff>